<commit_message>
Feat: Ambient 사운드 추가
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excel/Sound.xlsx
+++ b/Assets/Resources/Excel/Sound.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Woo_260126\UnityProject_LucidDiver\Assets\Resources\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED1A279-FFE7-4DAA-8C61-F94FF764D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85443220-68F4-49A3-9DEA-2E704BE852E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2145" yWindow="1185" windowWidth="21480" windowHeight="13380" xr2:uid="{390C7208-66F1-497C-8CC9-7C965485B0DB}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="76">
   <si>
     <t>AudioID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -273,6 +273,9 @@
   </si>
   <si>
     <t>Yuan_Memory</t>
+  </si>
+  <si>
+    <t>InGame_Embient_2</t>
   </si>
 </sst>
 </file>
@@ -636,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA92F57-20FC-47F2-9478-340152432242}">
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="23.625" bestFit="1" customWidth="1"/>
@@ -1122,13 +1125,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>10401</v>
+        <v>10306</v>
       </c>
       <c r="B29" t="s">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="C29" t="s">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1139,10 +1142,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>10402</v>
+        <v>10401</v>
       </c>
       <c r="B30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" t="s">
         <v>5</v>
@@ -1156,10 +1159,10 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>10403</v>
+        <v>10402</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C31" t="s">
         <v>5</v>
@@ -1168,15 +1171,15 @@
         <v>1</v>
       </c>
       <c r="E31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>10404</v>
+        <v>10403</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" t="s">
         <v>5</v>
@@ -1190,10 +1193,10 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>10501</v>
+        <v>10404</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
         <v>5</v>
@@ -1207,10 +1210,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>10502</v>
+        <v>10501</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C34" t="s">
         <v>5</v>
@@ -1224,10 +1227,10 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>10503</v>
+        <v>10502</v>
       </c>
       <c r="B35" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C35" t="s">
         <v>5</v>
@@ -1241,10 +1244,10 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>10504</v>
+        <v>10503</v>
       </c>
       <c r="B36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C36" t="s">
         <v>5</v>
@@ -1258,10 +1261,10 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>10505</v>
+        <v>10504</v>
       </c>
       <c r="B37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C37" t="s">
         <v>5</v>
@@ -1275,10 +1278,10 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>10506</v>
+        <v>10505</v>
       </c>
       <c r="B38" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C38" t="s">
         <v>5</v>
@@ -1292,10 +1295,10 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>10507</v>
+        <v>10506</v>
       </c>
       <c r="B39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C39" t="s">
         <v>5</v>
@@ -1309,10 +1312,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>10508</v>
+        <v>10507</v>
       </c>
       <c r="B40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C40" t="s">
         <v>5</v>
@@ -1326,10 +1329,10 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>10509</v>
+        <v>10508</v>
       </c>
       <c r="B41" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C41" t="s">
         <v>5</v>
@@ -1343,10 +1346,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>10510</v>
+        <v>10509</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C42" t="s">
         <v>5</v>
@@ -1360,10 +1363,10 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>10601</v>
+        <v>10510</v>
       </c>
       <c r="B43" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C43" t="s">
         <v>5</v>
@@ -1377,10 +1380,10 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>10602</v>
+        <v>10601</v>
       </c>
       <c r="B44" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C44" t="s">
         <v>5</v>
@@ -1394,44 +1397,44 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45">
-        <v>10603</v>
+        <v>10602</v>
       </c>
       <c r="B45" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C45" t="s">
         <v>5</v>
       </c>
       <c r="D45">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="E45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46">
-        <v>10701</v>
+        <v>10603</v>
       </c>
       <c r="B46" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C46" t="s">
         <v>5</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>10702</v>
+        <v>10701</v>
       </c>
       <c r="B47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C47" t="s">
         <v>5</v>
@@ -1445,10 +1448,10 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>10703</v>
+        <v>10702</v>
       </c>
       <c r="B48" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C48" t="s">
         <v>5</v>
@@ -1462,10 +1465,10 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>10704</v>
+        <v>10703</v>
       </c>
       <c r="B49" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C49" t="s">
         <v>5</v>
@@ -1479,10 +1482,10 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50">
-        <v>10705</v>
+        <v>10704</v>
       </c>
       <c r="B50" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C50" t="s">
         <v>5</v>
@@ -1496,10 +1499,10 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>10706</v>
+        <v>10705</v>
       </c>
       <c r="B51" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C51" t="s">
         <v>5</v>
@@ -1513,10 +1516,10 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>10801</v>
+        <v>10706</v>
       </c>
       <c r="B52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C52" t="s">
         <v>5</v>
@@ -1525,32 +1528,32 @@
         <v>1</v>
       </c>
       <c r="E52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>10901</v>
+        <v>10801</v>
       </c>
       <c r="B53" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="C53" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D53">
         <v>1</v>
       </c>
       <c r="E53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>10902</v>
+        <v>10901</v>
       </c>
       <c r="B54" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C54" t="s">
         <v>6</v>
@@ -1564,10 +1567,10 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>10903</v>
+        <v>10902</v>
       </c>
       <c r="B55" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C55" t="s">
         <v>6</v>
@@ -1581,10 +1584,10 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>10904</v>
+        <v>10903</v>
       </c>
       <c r="B56" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C56" t="s">
         <v>6</v>
@@ -1598,10 +1601,10 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>10905</v>
+        <v>10904</v>
       </c>
       <c r="B57" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C57" t="s">
         <v>6</v>
@@ -1615,10 +1618,10 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>10906</v>
+        <v>10905</v>
       </c>
       <c r="B58" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C58" t="s">
         <v>6</v>
@@ -1632,10 +1635,10 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>10907</v>
+        <v>10906</v>
       </c>
       <c r="B59" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C59" t="s">
         <v>6</v>
@@ -1649,10 +1652,10 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>10908</v>
+        <v>10907</v>
       </c>
       <c r="B60" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C60" t="s">
         <v>6</v>
@@ -1666,10 +1669,10 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>10909</v>
+        <v>10908</v>
       </c>
       <c r="B61" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C61" t="s">
         <v>6</v>
@@ -1683,13 +1686,13 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>11001</v>
+        <v>10909</v>
       </c>
       <c r="B62" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="C62" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D62">
         <v>1</v>
@@ -1700,10 +1703,10 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>11002</v>
+        <v>11001</v>
       </c>
       <c r="B63" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C63" t="s">
         <v>5</v>
@@ -1717,10 +1720,10 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>11003</v>
+        <v>11002</v>
       </c>
       <c r="B64" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C64" t="s">
         <v>5</v>
@@ -1734,10 +1737,10 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>11004</v>
+        <v>11003</v>
       </c>
       <c r="B65" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C65" t="s">
         <v>5</v>
@@ -1751,10 +1754,10 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>11005</v>
+        <v>11004</v>
       </c>
       <c r="B66" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C66" t="s">
         <v>5</v>
@@ -1768,18 +1771,35 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67">
+        <v>11005</v>
+      </c>
+      <c r="B67" t="s">
+        <v>63</v>
+      </c>
+      <c r="C67" t="s">
+        <v>5</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+      <c r="E67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A68">
         <v>11006</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B68" t="s">
         <v>64</v>
       </c>
-      <c r="C67" t="s">
-        <v>5</v>
-      </c>
-      <c r="D67">
-        <v>1</v>
-      </c>
-      <c r="E67" t="b">
+      <c r="C68" t="s">
+        <v>5</v>
+      </c>
+      <c r="D68">
+        <v>1</v>
+      </c>
+      <c r="E68" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>